<commit_message>
Transitioned from Plan to Build mode
Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6c2e3097-ead6-4eab-86a7-40c33b3aa100
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/PyJNGyq
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-01.xlsx
+++ b/backups/proposal-log-2026-04-01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="81">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -136,7 +136,7 @@
     <t>Inglewood Transit Connector RFQ</t>
   </si>
   <si>
-    <t>TM (LAX)</t>
+    <t>LAX - FS</t>
   </si>
   <si>
     <t>Retail</t>
@@ -199,7 +199,7 @@
     <t>FINN Partners at First &amp; Main</t>
   </si>
   <si>
-    <t>Portland (PDX)</t>
+    <t>CLT - S Carolina</t>
   </si>
   <si>
     <t>Aviation</t>
@@ -214,6 +214,12 @@
     <t>Automated Lead</t>
   </si>
   <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>Submitted</t>
+  </si>
+  <si>
     <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
   </si>
   <si>
@@ -229,6 +235,9 @@
     <t>Joseph Dinielli</t>
   </si>
   <si>
+    <t>Notes for the project.</t>
+  </si>
+  <si>
     <t>https://app.buildingconnected.com/opportunities/69cd0562786a720050b13b93</t>
   </si>
   <si>
@@ -242,6 +251,9 @@
   </si>
   <si>
     <t>2026-07-30</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cd0562786a720050b13b93/info</t>
   </si>
 </sst>
 </file>
@@ -990,10 +1002,10 @@
         <v>66</v>
       </c>
       <c r="I8" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="J8" t="s">
-        <v>22</v>
+        <v>68</v>
       </c>
       <c r="K8" t="s">
         <v>20</v>
@@ -1005,15 +1017,15 @@
         <v>20</v>
       </c>
       <c r="N8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -1025,13 +1037,13 @@
         <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I9" t="s">
         <v>20</v>
@@ -1046,21 +1058,21 @@
         <v>20</v>
       </c>
       <c r="M9" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="N9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
         <v>17</v>
@@ -1069,7 +1081,7 @@
         <v>64</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1084,16 +1096,16 @@
         <v>22</v>
       </c>
       <c r="K10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="L10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="M10" t="s">
         <v>20</v>
       </c>
       <c r="N10" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correctly display region names in proposals and logs
Fix hardcoded "EXT - External" display for regions across the frontend (ProjectLogPage.tsx, public/tools/proposal-log.html) and backend (server/regionMatcher.ts) to show the actual region names.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: ae8744eb-d4a5-4c9e-8181-a709cc579bb0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/4UbUBjw
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-01.xlsx
+++ b/backups/proposal-log-2026-04-01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -53,6 +53,105 @@
   </si>
   <si>
     <t>BC Link</t>
+  </si>
+  <si>
+    <t>26-0199</t>
+  </si>
+  <si>
+    <t>Arrowhead Regional Med Ctr. (ARMC) DB PS (REBID)</t>
+  </si>
+  <si>
+    <t>LAX</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>Gabriel Frota</t>
+  </si>
+  <si>
+    <t>No Bid</t>
+  </si>
+  <si>
+    <t>Automated test note</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6f855787ef64d5cc05edb</t>
+  </si>
+  <si>
+    <t>26-0196</t>
+  </si>
+  <si>
+    <t>Univ of Oregon - Esslinger Hall Re-roof</t>
+  </si>
+  <si>
+    <t>PDX</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>Mark Socks</t>
+  </si>
+  <si>
+    <t>Lost</t>
+  </si>
+  <si>
+    <t>NO BID - No Scope</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c1b75e4cb9ae021994a5b7</t>
+  </si>
+  <si>
+    <t>26-0194</t>
+  </si>
+  <si>
+    <t>FINN Partners at First &amp; Main</t>
+  </si>
+  <si>
+    <t>CLT - S Carolina</t>
+  </si>
+  <si>
+    <t>Aviation</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>Automated Lead</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>Submitted</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69bc538e7aaadb003896155f</t>
+  </si>
+  <si>
+    <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
+  </si>
+  <si>
+    <t>SEA - Washington</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>Merci Keathley</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
   </si>
 </sst>
 </file>
@@ -451,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -511,8 +610,184 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" t="s">
+        <v>17</v>
+      </c>
+      <c r="M3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>45</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L5" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N5" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:N5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Make the Self Perform Estimator field editable in the proposal log
Add 'selfPerformEstimator' field to proposal log schema, service layer, API routes, and frontend to allow inline editing and data synchronization.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 35814072-4f37-45f0-838f-90097c00cdbe
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/8T9SOcd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-01.xlsx
+++ b/backups/proposal-log-2026-04-01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -142,10 +142,13 @@
     <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
   </si>
   <si>
-    <t>SEA - Washington</t>
+    <t>ATL - Atlanta</t>
   </si>
   <si>
     <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>HK</t>
   </si>
   <si>
     <t>Merci Keathley</t>
@@ -762,10 +765,10 @@
         <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I5" t="s">
         <v>17</v>
@@ -783,7 +786,7 @@
         <v>17</v>
       </c>
       <c r="N5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>